<commit_message>
darn it forgot to update familiarity
</commit_message>
<xml_diff>
--- a/01-Translation/task_translation_template.xlsx
+++ b/01-Translation/task_translation_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erinbuchanan/GitHub/Research/2_projects/ManyLanguages-Grant/ML-One-Network/01-Translation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05FB3F42-D375-FA41-B9BD-A3989CC14080}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3E85294-0BA7-2F4A-A734-734B2284983A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -687,12 +687,6 @@
     <t>Please work at a rapid place and don't spend too much time thinking about each word. Rather, make your ratings based on your first and immediate reaction as you read each word. If you do not know the word presented, please select X.</t>
   </si>
   <si>
-    <t>In the following pages, you will see a series of target words. Your task is to rate how familiar or known each word is to you. If a word feels very familiar or well known, select 9 on the scale; if it feels hardly familiar or unknown, select 1. The numbers from 1 to 9 represent increasing levels of familiarity. Please choose the number that best reflects your experience with each word.</t>
-  </si>
-  <si>
-    <t>Please rate the familarity of each word from 1 (unknown, very unfamiliar) to 9 (well known, very familiar). Please choose the number that best reflects your experience with each word.</t>
-  </si>
-  <si>
     <t>For each word, rate arousal (1 = very calm/relaxed, 9 = very excited/activated). If you do not know the word, leave the rating blank and mark X below.</t>
   </si>
   <si>
@@ -760,6 +754,12 @@
   </si>
   <si>
     <t>English</t>
+  </si>
+  <si>
+    <t>Please rate the familarity of each word from 1 (unknown, very unfamiliar) to 9 (well known, very familiar).</t>
+  </si>
+  <si>
+    <t>In the following pages, you will see a series of target words. Your task is to rate how familiar or known each word is to you. If a word feels very familiar or well known, select 9 on the scale; if it feels hardly familiar or unknown, select 1. The numbers from 1 to 9 represent increasing levels of familiarity.</t>
   </si>
 </sst>
 </file>
@@ -1157,7 +1157,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1167,7 +1167,7 @@
     </row>
     <row r="3" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="102" x14ac:dyDescent="0.2">
@@ -1197,7 +1197,7 @@
     </row>
     <row r="9" spans="1:1" ht="170" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1217,7 +1217,7 @@
     </row>
     <row r="13" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1297,7 +1297,7 @@
     </row>
     <row r="29" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="30" spans="1:1" ht="34" x14ac:dyDescent="0.2">
@@ -1310,14 +1310,14 @@
         <v>77</v>
       </c>
     </row>
-    <row r="32" spans="1:1" ht="51" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>169</v>
+        <v>191</v>
       </c>
     </row>
     <row r="33" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="34" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1350,14 +1350,14 @@
         <v>59</v>
       </c>
     </row>
-    <row r="40" spans="1:1" ht="85" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:1" ht="68" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>168</v>
+        <v>192</v>
       </c>
     </row>
     <row r="41" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="42" spans="1:1" ht="68" x14ac:dyDescent="0.2">
@@ -1392,12 +1392,12 @@
     </row>
     <row r="48" spans="1:1" ht="102" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="49" spans="1:1" ht="136" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="50" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1407,12 +1407,12 @@
     </row>
     <row r="51" spans="1:1" ht="68" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="52" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="53" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1447,7 +1447,7 @@
     </row>
     <row r="59" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="60" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1542,7 +1542,7 @@
     </row>
     <row r="78" spans="1:1" ht="68" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="79" spans="1:1" ht="34" x14ac:dyDescent="0.2">
@@ -1562,7 +1562,7 @@
     </row>
     <row r="82" spans="1:1" ht="68" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="83" spans="1:1" ht="34" x14ac:dyDescent="0.2">
@@ -1597,7 +1597,7 @@
     </row>
     <row r="89" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="90" spans="1:1" ht="170" x14ac:dyDescent="0.2">
@@ -1637,7 +1637,7 @@
     </row>
     <row r="97" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="98" spans="1:1" ht="85" x14ac:dyDescent="0.2">
@@ -1657,37 +1657,37 @@
     </row>
     <row r="101" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A101" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="102" spans="1:1" ht="136" x14ac:dyDescent="0.2">
       <c r="A102" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="103" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A103" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="104" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A104" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="105" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A105" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="106" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A106" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="107" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A107" s="2" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
add new "click finish!" translation
</commit_message>
<xml_diff>
--- a/01-Translation/task_translation_template.xlsx
+++ b/01-Translation/task_translation_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erinbuchanan/GitHub/Research/2_projects/ManyLanguages-Grant/ML-One-Network/01-Translation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19AA3C9E-D844-CF49-83F6-D396E2351178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D91E0936-A7FB-F842-81D0-63D2D196DB57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="194">
   <si>
     <t>Thank you</t>
   </si>
@@ -760,6 +760,9 @@
   </si>
   <si>
     <t>Please rate the familiarity of each word from 1 (unknown, very unfamiliar) to 9 (well known, very familiar).</t>
+  </si>
+  <si>
+    <t>Important: You must click Finish to submit your responses and receive credit or payment.</t>
   </si>
 </sst>
 </file>
@@ -1390,7 +1393,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="48" spans="1:1" ht="102" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:1" ht="119" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>173</v>
       </c>
@@ -1690,8 +1693,10 @@
         <v>180</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A108"/>
+    <row r="108" spans="1:1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A108" s="2" t="s">
+        <v>193</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:B100">

</xml_diff>

<commit_message>
try updating translation template
</commit_message>
<xml_diff>
--- a/01-Translation/task_translation_template.xlsx
+++ b/01-Translation/task_translation_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erinbuchanan/GitHub/Research/2_projects/ManyLanguages-Grant/ML-One-Network/01-Translation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2038726F-E226-334E-8FC5-425404DA0F65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87689DDC-A157-6B40-9EC0-4A17BF955F20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4740" yWindow="2380" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="aoa" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="188">
   <si>
     <t>Thank you</t>
   </si>
@@ -66,9 +66,6 @@
     <t>Background Information:</t>
   </si>
   <si>
-    <t>In this study, you will be asked to complete different questions about word concepts. For example, you may be asked to define a word’s characteristics, rate how familiar you are with a word, or simply judge if a string of letters is a real word.</t>
-  </si>
-  <si>
     <t>Procedures:</t>
   </si>
   <si>
@@ -171,9 +168,6 @@
     <t>How to do this task</t>
   </si>
   <si>
-    <t>Please rate the following words by entering the age in years at which you think you learned the word. An approximate age is good enough for this rating.</t>
-  </si>
-  <si>
     <t>Word ratings</t>
   </si>
   <si>
@@ -183,9 +177,6 @@
     <t>For each word, enter the age (in years) when you think you learned it, or select X if unknown.</t>
   </si>
   <si>
-    <t>Enter an age or select X.</t>
-  </si>
-  <si>
     <t>Enter a whole number from 1 to 100.</t>
   </si>
   <si>
@@ -228,9 +219,6 @@
     <t>Please rate the following words by entering the age in years at which you think you learned the word. An approximate age is good enough for this rating</t>
   </si>
   <si>
-    <t>If you do not know the word, please select the letter X.</t>
-  </si>
-  <si>
     <t>Word ratings (Block ${blockIndex + 1} of ${wordBlocks.length})</t>
   </si>
   <si>
@@ -246,37 +234,19 @@
     <t>Some words refer to things or actions in reality, which you can experience directly through one of the five senses. We call these words concrete words. Other words refer to meanings that cannot be experienced directly but which we know because the meanings can be defined by other words. These are abstract words. Still other words fall in-between the two extremes, because we can experience them to some extent; and in addition, we rely on language to understand them. We want you to indicate how concrete the meaning of each word is for you by using a 9-point rating scale going from abstract to concrete. A concrete word comes with a higher rating and refers to something that exists in reality; you can have immediate experience of it through your senses (smelling, tasting, touching, hearing, seeing) and the actions you do.</t>
   </si>
   <si>
-    <t>The easiest way to explain a word is by pointing to it or by demonstrating it (e.g. To explain 'sweet' you could have someone eat sugar; To explain 'jump' you could simply jump up and down or show people a movie clip about someone jumping up and down; To explain 'couch', you could point to a couch or show a picture of a couch). An abstract word comes with a lower rating and refers to something you cannot experience directly through your senses or actions. Its meaning depends on language. The easiest way to explain it is by using other words (e.g. There is no simple way to demonstrate 'justice'; but we can explain the meaning of the word by using other words that capture parts of its meaning).</t>
-  </si>
-  <si>
     <t>Always think of how concrete (experience based) the meaning of the word is to you. In all likelihood, you will encounter several words you do not know well enough to give a useful rating. This is informative to us too, as in our research we only want to use words known to people. We may also include one or two fake words which cannot be known by you. Please indicate when you don't know a word by using the letter X.</t>
   </si>
   <si>
-    <t>For each word, rate how abstract (1) or concrete (9) it feels. If you do not know the word, leave the rating blank and mark X below.</t>
-  </si>
-  <si>
-    <t>Rating (1 = very abstract, 9 = very concrete)</t>
-  </si>
-  <si>
     <t>Rating (1 = very unfamiliar, 9 = very familiar)</t>
   </si>
   <si>
     <t>This is an experiment to find out how easy or difficult it is to imagine a mental picture of the word presented to you. You will be given a list of words, and you are to rate each one from how easy it is to picture the word (apple; high imagery) to words that may not be imagined easily (fact; low imagery).</t>
   </si>
   <si>
-    <t>For each word, rate how difficult (1) or easy (9) it is to imagine a mental picture of the object. If you do not know the word, leave the rating blank and mark X below.</t>
-  </si>
-  <si>
-    <t>Rating (1 = very difficult, 9 = very easy)</t>
-  </si>
-  <si>
     <t>The top panel shows the happy-unhappy scale, which ranges from a frown to a smile. At one extreme of this scale, you are happy, pleased, satisfied, contented, hopeful. When you feel completely happy you should indicate this by selecting the 9 on the right. The other end of the scale is when you feel completely unhappy, annoyed, unsatisfied, melancholic, despaired, or bored. You can indicate feeling completely unhappy by selecting the 1 on the left. The figures also allow you to describe intermediate feelings of pleasure, by selecting any values in the middle. If you feel completely neutral, neither happy nor sad, select the 4 in the middle.</t>
   </si>
   <si>
     <t>Valence ratings (Block ${blockIndex + 1} of ${wordBlocks.length})</t>
-  </si>
-  <si>
-    <t>Rating (1 = very unpleasant/unhappy, 9 = very pleasant/happy)</t>
   </si>
   <si>
     <t>concrete</t>
@@ -678,15 +648,6 @@
     <t>Arousal ratings</t>
   </si>
   <si>
-    <t>We call this set of figures SAM, and you will be using these figures to rate how you feel while reading each word. The picture shows the unhappy-happy scale, which ranges from a frown to a smile. At one extreme of this scale, you are happy, pleased, satisfied, contented, hopeful. When you feel completely happy you should indicate this by selecting the 9 on the right. The other end of the scale is when you feel completely unhappy, annoyed, unsatisfied, melancholic, despaired, or bored. You can indicate feeling completely unhappy by selecting the 1 on the left. The figures also allow you to describe intermediate feelings of pleasure, by selecting any values in the middle. If you feel completely neutral, neither happy nor sad, select the 4 in the middle.</t>
-  </si>
-  <si>
-    <t>Please work at a rapid place and don't spend too much time thinking about each word. Rather, make your ratings based on your first and immediate reaction as you read each word. If you do not know the word presented, please select X.</t>
-  </si>
-  <si>
-    <t>For each word, rate valence (1 = very unpleasant/unhappy, 9 = very pleasant/happy). If you do not know the word, leave the rating blank and mark X below.</t>
-  </si>
-  <si>
     <t>We call this set of figures SAM, and you will be using these figures to rate how you feel while reading each word. The picture shows the unhappy-happy scale, which ranges from a frown to a smile. At one extreme of this scale, you feel completely unhappy, annoyed, unsatisfied, melancholic, despaired, or bored. You can indicate feeling completely unhappy by selecting the 1 on the left. The other end of the scale, you feel happy, pleased, satisfied, contented, or hopeful. When you feel completely happy you should indicate this by selecting the 9 on the right. The figures also allow you to describe intermediate feelings of pleasure, by selecting any values in the middle. If you feel completely neutral, neither happy nor sad, select the 4 in the middle.</t>
   </si>
   <si>
@@ -732,18 +693,12 @@
     <t>At one extreme of this scale you would feel completely relaxed, calm, sluggish, dull, sleepy, or unaroused. Indicate feeling calm by selecting the 1 on the left.  Now look at the other end of the calm-excited scale, which is the completely opposite feeling. You would feel stimulated, excited, frenzied, jittery, wide-awake, or aroused. When you feel completely aroused, select the 9 on the right. The figures also allow you to describe intermediate feelings of calmness or excitedness by selecting any other number. If you are not excited nor at all calm, select the 4 in the middle.</t>
   </si>
   <si>
-    <t>Please work at a rapid place and don't spend too much time thinking about each word. Rather, make your ratings based on your first and immediate reaction as you read each word.</t>
-  </si>
-  <si>
     <t>Self-Assessment Manikin (SAM) scale for arousal</t>
   </si>
   <si>
     <t>Please select a rating or mark unknown</t>
   </si>
   <si>
-    <t>Please select a rating for every word</t>
-  </si>
-  <si>
     <t>Self-Assessment Manikin (SAM) scale for valence</t>
   </si>
   <si>
@@ -753,13 +708,43 @@
     <t>In the following pages, you will see a series of target words. Your task is to rate how familiar or known each word is to you. If a word feels very familiar or well known, select 9 on the scale; if it feels hardly familiar or unknown, select 1. The numbers from 1 to 9 represent increasing levels of familiarity.</t>
   </si>
   <si>
-    <t>Please rate the familiarity of each word from 1 (unknown, very unfamiliar) to 9 (well known, very familiar).</t>
-  </si>
-  <si>
     <t>Important: You must click Finish to submit your responses and receive credit or payment.</t>
   </si>
   <si>
     <t xml:space="preserve">Rating (1 = very calm/relaxed, 9 = very excited/activated) or X (Unknown) </t>
+  </si>
+  <si>
+    <t>The easiest way to explain a word is by pointing to it or by demonstrating it (e.g., To explain 'sweet' you could have someone eat sugar; To explain 'jump' you could simply jump up and down or show people a movie clip about someone jumping up and down; To explain 'couch', you could point to a couch or show a picture of a couch). An abstract word comes with a lower rating and refers to something you cannot experience directly through your senses or actions. Its meaning depends on language. The easiest way to explain it is by using other words (e.g., There is no simple way to demonstrate 'justice'; but we can explain the meaning of the word by using other words that capture parts of its meaning).</t>
+  </si>
+  <si>
+    <t>Rating (1 = very abstract, 9 = very concrete) or X (Unknown)</t>
+  </si>
+  <si>
+    <t>Please select a rating</t>
+  </si>
+  <si>
+    <t>Rating (1 = very difficult to imagine, 9 = very easy to imagine) or X (Unknown)</t>
+  </si>
+  <si>
+    <t>Age ratings</t>
+  </si>
+  <si>
+    <t>Enter an age or select unknown.</t>
+  </si>
+  <si>
+    <t>If you do not know the word, please select the letter X for unknown.</t>
+  </si>
+  <si>
+    <t>Imagination ratings</t>
+  </si>
+  <si>
+    <t>Emotion ratings</t>
+  </si>
+  <si>
+    <t>Rating (1 = very unpleasant/unhappy, 9 = very pleasant/happy) or X (Unknown)</t>
+  </si>
+  <si>
+    <t>Please work at a rapid pace and don't spend too much time thinking about each word. Rather, make your ratings based on your first and immediate reaction as you read each word. If you do not know the word, please select the letter X for unknown.</t>
   </si>
 </sst>
 </file>
@@ -1146,10 +1131,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A107"/>
+  <dimension ref="A1:A104"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="66.1640625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="86.33203125" style="2" customWidth="1"/>
     <col min="2" max="2" width="76" style="2" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" style="2" customWidth="1"/>
     <col min="4" max="16384" width="10.83203125" style="2"/>
@@ -1157,542 +1142,520 @@
   <sheetData>
     <row r="1" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>188</v>
+        <v>173</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>47</v>
+        <v>168</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="102" x14ac:dyDescent="0.2">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>71</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>41</v>
+        <v>166</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="68" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" ht="170" x14ac:dyDescent="0.2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>168</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" ht="102" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" ht="51" x14ac:dyDescent="0.2">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>174</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" ht="102" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>15</v>
+        <v>161</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
-        <v>5</v>
+      <c r="A18" s="2" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A22" s="2" t="s">
-        <v>39</v>
+      <c r="A22" s="3" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>50</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>58</v>
+        <v>21</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" ht="34" x14ac:dyDescent="0.2">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
         <v>48</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A29" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A30" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A31" s="2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A32" s="2" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="33" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
     </row>
     <row r="34" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
     </row>
     <row r="35" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>23</v>
+        <v>43</v>
       </c>
     </row>
     <row r="36" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="37" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>64</v>
+        <v>23</v>
       </c>
     </row>
     <row r="38" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" ht="68" x14ac:dyDescent="0.2">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" ht="51" x14ac:dyDescent="0.2">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="41" spans="1:1" ht="68" x14ac:dyDescent="0.2">
-      <c r="A41" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" ht="68" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>34</v>
+        <v>58</v>
       </c>
     </row>
     <row r="45" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
     </row>
     <row r="46" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" ht="119" x14ac:dyDescent="0.2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" ht="136" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" ht="85" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" ht="68" x14ac:dyDescent="0.2">
-      <c r="A50" s="2" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="51" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
-        <v>170</v>
+        <v>156</v>
       </c>
     </row>
     <row r="52" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="53" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="54" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="55" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="56" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" ht="34" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
-        <v>45</v>
+        <v>179</v>
       </c>
     </row>
     <row r="58" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
-        <v>185</v>
+        <v>171</v>
       </c>
     </row>
     <row r="59" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="60" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="61" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="62" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
-        <v>166</v>
+        <v>187</v>
       </c>
     </row>
     <row r="63" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="64" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="65" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="66" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
-        <v>73</v>
+        <v>178</v>
       </c>
     </row>
     <row r="67" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
-        <v>192</v>
+        <v>176</v>
       </c>
     </row>
     <row r="68" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
-        <v>77</v>
+        <v>180</v>
       </c>
     </row>
     <row r="69" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
     </row>
     <row r="70" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
-        <v>80</v>
+        <v>186</v>
       </c>
     </row>
     <row r="71" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="72" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1" ht="187" x14ac:dyDescent="0.2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
-        <v>69</v>
+        <v>170</v>
       </c>
     </row>
     <row r="74" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" ht="153" x14ac:dyDescent="0.2">
+      <c r="A75" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A76" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A75" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="76" spans="1:1" ht="153" x14ac:dyDescent="0.2">
-      <c r="A76" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="77" spans="1:1" ht="68" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="78" spans="1:1" ht="34" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" ht="119" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="79" spans="1:1" ht="153" x14ac:dyDescent="0.2">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A79" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="80" spans="1:1" ht="68" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="81" spans="1:1" ht="68" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" ht="119" x14ac:dyDescent="0.2">
       <c r="A81" s="2" t="s">
-        <v>173</v>
+        <v>69</v>
       </c>
     </row>
     <row r="82" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A83" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A84" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A85" s="2" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="83" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A83" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="84" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A84" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="85" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A85" s="2" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="86" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
-        <v>60</v>
+        <v>6</v>
       </c>
     </row>
     <row r="87" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="88" spans="1:1" ht="51" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="89" spans="1:1" ht="170" x14ac:dyDescent="0.2">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
-        <v>165</v>
+        <v>57</v>
       </c>
     </row>
     <row r="90" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A90" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="91" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" ht="136" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="92" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="93" spans="1:1" ht="51" x14ac:dyDescent="0.2">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A93" s="2" t="s">
-        <v>7</v>
+        <v>39</v>
       </c>
     </row>
     <row r="94" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
     </row>
     <row r="95" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A95" s="2" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="96" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="97" spans="1:1" ht="85" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="98" spans="1:1" ht="68" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
-        <v>19</v>
+        <v>50</v>
       </c>
     </row>
     <row r="99" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="100" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" ht="68" x14ac:dyDescent="0.2">
       <c r="A100" s="2" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="101" spans="1:1" ht="136" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A101" s="2" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="102" spans="1:1" ht="51" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A102" s="2" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="103" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A103" s="2" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="104" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A104" s="2" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="105" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A105" s="2" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="106" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A106" s="2" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="107" spans="1:1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A107" s="2" t="s">
-        <v>191</v>
-      </c>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A104"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:B99">
-    <sortCondition ref="A1:A99"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A103">
+    <sortCondition ref="A2:A103"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -1706,1784 +1669,1784 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:3" s="1" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>91</v>
-      </c>
       <c r="C8" s="2" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
     </row>
     <row r="16" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="17" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
     </row>
     <row r="18" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
     </row>
     <row r="19" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
     </row>
     <row r="20" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
     </row>
     <row r="21" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
     </row>
     <row r="23" spans="1:3" s="1" customFormat="1" ht="409" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
     </row>
     <row r="24" spans="1:3" s="1" customFormat="1" ht="238" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
     </row>
     <row r="25" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
     </row>
     <row r="26" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
     </row>
     <row r="27" spans="1:3" s="1" customFormat="1" ht="68" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
     </row>
     <row r="28" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
     </row>
     <row r="29" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
     </row>
     <row r="30" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
     </row>
     <row r="31" spans="1:3" s="1" customFormat="1" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
     </row>
     <row r="32" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
     </row>
     <row r="33" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
     </row>
     <row r="34" spans="1:3" s="1" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
     </row>
     <row r="35" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="36" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
     </row>
     <row r="38" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="40" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
     </row>
     <row r="41" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
     </row>
     <row r="42" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
     </row>
     <row r="43" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
     </row>
     <row r="44" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
     </row>
     <row r="45" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
     </row>
     <row r="46" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="47" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
     </row>
     <row r="48" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="49" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
     </row>
     <row r="50" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
     </row>
     <row r="51" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
     </row>
     <row r="52" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
     </row>
     <row r="53" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
     <row r="54" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
     </row>
     <row r="55" spans="1:3" s="1" customFormat="1" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
     </row>
     <row r="56" spans="1:3" s="1" customFormat="1" ht="238" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
     </row>
     <row r="57" spans="1:3" s="1" customFormat="1" ht="221" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
     </row>
     <row r="58" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
     </row>
     <row r="59" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="60" spans="1:3" s="1" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
     </row>
     <row r="61" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
     </row>
     <row r="62" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
     </row>
     <row r="63" spans="1:3" s="1" customFormat="1" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
     </row>
     <row r="64" spans="1:3" s="1" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B64" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B64" s="2" t="s">
-        <v>138</v>
-      </c>
       <c r="C64" s="2" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
     </row>
     <row r="65" spans="1:3" s="1" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
     </row>
     <row r="66" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
     </row>
     <row r="67" spans="1:3" s="1" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
     </row>
     <row r="68" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="69" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
     </row>
     <row r="70" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
     </row>
     <row r="71" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
     </row>
     <row r="72" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="73" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
     </row>
     <row r="74" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
     </row>
     <row r="75" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
     </row>
     <row r="76" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
     </row>
     <row r="77" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
     </row>
     <row r="78" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
     </row>
     <row r="79" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="80" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
     </row>
     <row r="81" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="82" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
     </row>
     <row r="83" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
     </row>
     <row r="84" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
     </row>
     <row r="85" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
     </row>
     <row r="86" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
     <row r="87" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
     </row>
     <row r="88" spans="1:3" s="1" customFormat="1" ht="170" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
     </row>
     <row r="89" spans="1:3" s="1" customFormat="1" ht="238" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
     </row>
     <row r="90" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
     </row>
     <row r="91" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
     </row>
     <row r="92" spans="1:3" s="1" customFormat="1" ht="68" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
     </row>
     <row r="93" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
     </row>
     <row r="94" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
     </row>
     <row r="95" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
     </row>
     <row r="96" spans="1:3" s="1" customFormat="1" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
     </row>
     <row r="97" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
     </row>
     <row r="98" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
     </row>
     <row r="99" spans="1:3" s="1" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
     </row>
     <row r="100" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="101" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
     </row>
     <row r="102" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
     </row>
     <row r="103" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
     </row>
     <row r="104" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="105" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
     </row>
     <row r="106" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
     </row>
     <row r="107" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
     </row>
     <row r="108" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
     </row>
     <row r="109" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
     </row>
     <row r="110" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
     </row>
     <row r="111" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="112" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
     </row>
     <row r="113" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="114" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
     </row>
     <row r="115" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
     </row>
     <row r="116" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
     </row>
     <row r="117" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
     </row>
     <row r="118" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
     <row r="119" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
     </row>
     <row r="120" spans="1:3" s="1" customFormat="1" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
     </row>
     <row r="121" spans="1:3" s="1" customFormat="1" ht="238" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
     </row>
     <row r="122" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
     </row>
     <row r="123" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
     </row>
     <row r="124" spans="1:3" s="1" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
     </row>
     <row r="125" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
     </row>
     <row r="126" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
     </row>
     <row r="127" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
     </row>
     <row r="128" spans="1:3" s="1" customFormat="1" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
     </row>
     <row r="129" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
     </row>
     <row r="130" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
     </row>
     <row r="131" spans="1:3" s="1" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
     </row>
     <row r="132" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B132" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="133" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B133" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
     </row>
     <row r="134" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B134" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
     </row>
     <row r="135" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B135" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
     </row>
     <row r="136" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="137" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
     </row>
     <row r="138" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
     </row>
     <row r="139" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
     </row>
     <row r="140" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
     </row>
     <row r="141" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
     </row>
     <row r="142" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
     </row>
     <row r="143" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="144" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
     </row>
     <row r="145" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="146" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
     </row>
     <row r="147" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
     </row>
     <row r="148" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
     </row>
     <row r="149" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
     </row>
     <row r="150" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
     <row r="151" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
     </row>
     <row r="152" spans="1:3" s="1" customFormat="1" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
     </row>
     <row r="153" spans="1:3" s="1" customFormat="1" ht="238" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
     </row>
     <row r="154" spans="1:3" s="1" customFormat="1" ht="221" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
     </row>
     <row r="155" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B155" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
     </row>
     <row r="156" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
     </row>
     <row r="157" spans="1:3" s="1" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
     </row>
     <row r="158" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
     </row>
     <row r="159" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
     </row>
     <row r="160" spans="1:3" s="1" customFormat="1" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
     </row>
     <row r="161" spans="1:3" s="1" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
     </row>
     <row r="162" spans="1:3" s="1" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding priming task to the translation pipeline
</commit_message>
<xml_diff>
--- a/01-Translation/task_translation_template.xlsx
+++ b/01-Translation/task_translation_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erinbuchanan/GitHub/Research/2_projects/ManyLanguages-Grant/ML-One-Network/01-Translation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8471F3AF-FE17-9640-9275-57BFB45AE7E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE54B976-BFFD-1140-9797-E21227E8B6D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4740" yWindow="2380" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="aoa" sheetId="1" r:id="rId1"/>
@@ -174,9 +174,6 @@
     <t>Age</t>
   </si>
   <si>
-    <t>For each word, enter the age (in years) when you think you learned it, or select X if unknown.</t>
-  </si>
-  <si>
     <t>Enter a whole number from 1 to 100.</t>
   </si>
   <si>
@@ -229,9 +226,6 @@
   </si>
   <si>
     <t>Some words refer to things or actions in reality, which you can experience directly through one of the five senses. We call these words concrete words. Other words refer to meanings that cannot be experienced directly but which we know because the meanings can be defined by other words. These are abstract words. Still other words fall in-between the two extremes, because we can experience them to some extent; and in addition, we rely on language to understand them. We want you to indicate how concrete the meaning of each word is for you by using a 9-point rating scale going from abstract to concrete. A concrete word comes with a higher rating and refers to something that exists in reality; you can have immediate experience of it through your senses (smelling, tasting, touching, hearing, seeing) and the actions you do.</t>
-  </si>
-  <si>
-    <t>Always think of how concrete (experience based) the meaning of the word is to you. In all likelihood, you will encounter several words you do not know well enough to give a useful rating. This is informative to us too, as in our research we only want to use words known to people. We may also include one or two fake words which cannot be known by you. Please indicate when you don't know a word by using the letter X.</t>
   </si>
   <si>
     <t>This is an experiment to find out how easy or difficult it is to imagine a mental picture of the word presented to you. You will be given a list of words, and you are to rate each one from how easy it is to picture the word (apple; high imagery) to words that may not be imagined easily (fact; low imagery).</t>
@@ -699,24 +693,12 @@
     <t>Important: You must click Finish to submit your responses and receive credit or payment.</t>
   </si>
   <si>
-    <t xml:space="preserve">Rating (1 = very calm/relaxed, 9 = very excited/activated) or X (Unknown) </t>
-  </si>
-  <si>
     <t>The easiest way to explain a word is by pointing to it or by demonstrating it (e.g., To explain 'sweet' you could have someone eat sugar; To explain 'jump' you could simply jump up and down or show people a movie clip about someone jumping up and down; To explain 'couch', you could point to a couch or show a picture of a couch). An abstract word comes with a lower rating and refers to something you cannot experience directly through your senses or actions. Its meaning depends on language. The easiest way to explain it is by using other words (e.g., There is no simple way to demonstrate 'justice'; but we can explain the meaning of the word by using other words that capture parts of its meaning).</t>
   </si>
   <si>
-    <t>Rating (1 = very abstract, 9 = very concrete) or X (Unknown)</t>
-  </si>
-  <si>
-    <t>Rating (1 = very difficult to imagine, 9 = very easy to imagine) or X (Unknown)</t>
-  </si>
-  <si>
     <t>Age ratings</t>
   </si>
   <si>
-    <t>Enter an age or select unknown.</t>
-  </si>
-  <si>
     <t>If you do not know the word, please select the letter X for unknown.</t>
   </si>
   <si>
@@ -726,9 +708,6 @@
     <t>Emotion ratings</t>
   </si>
   <si>
-    <t>Rating (1 = very unpleasant/unhappy, 9 = very pleasant/happy) or X (Unknown)</t>
-  </si>
-  <si>
     <t>Begin</t>
   </si>
   <si>
@@ -754,6 +733,27 @@
   </si>
   <si>
     <t>(Block ${PAGE_INDEX + 1} of ${TOTAL_TASK_PAGES})</t>
+  </si>
+  <si>
+    <t>Rating (1 = very abstract, 9 = very concrete) or X (Don't know the word)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rating (1 = very calm/relaxed, 9 = very excited/activated) or X (Don't know the word) </t>
+  </si>
+  <si>
+    <t>Rating (1 = very difficult to imagine, 9 = very easy to imagine) or X (Don't know the word)</t>
+  </si>
+  <si>
+    <t>Rating (1 = very unpleasant/unhappy, 9 = very pleasant/happy) or X (Don't know the word)</t>
+  </si>
+  <si>
+    <t>Always think of how concrete (experience based) the meaning of the word is to you. In all likelihood, you will encounter several words you do not know well enough to give a useful rating. This is informative to us too, as in our research we only want to use words known to people. We may also include one or two fake words which cannot be known by you. If you do not know the word, please select the letter X for unknown.</t>
+  </si>
+  <si>
+    <t>Enter an age or if you do not know the word, please select the letter X for unknown.</t>
+  </si>
+  <si>
+    <t>For each word, enter the age (in years) when you think you learned it. An approximate age is good enough for this rating. If you do not know the word, please select the letter X for unknown.</t>
   </si>
 </sst>
 </file>
@@ -1151,17 +1151,17 @@
   <sheetData>
     <row r="1" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1171,17 +1171,17 @@
     </row>
     <row r="5" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="68" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>65</v>
+        <v>188</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1191,12 +1191,12 @@
     </row>
     <row r="9" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1206,7 +1206,7 @@
     </row>
     <row r="12" spans="1:1" ht="102" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1226,12 +1226,12 @@
     </row>
     <row r="16" spans="1:1" ht="102" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1246,7 +1246,7 @@
     </row>
     <row r="20" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1281,22 +1281,22 @@
     </row>
     <row r="27" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
     </row>
     <row r="30" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="31" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1306,12 +1306,12 @@
     </row>
     <row r="32" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>46</v>
+        <v>190</v>
       </c>
     </row>
     <row r="34" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1336,37 +1336,37 @@
     </row>
     <row r="38" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
     </row>
     <row r="39" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="40" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
     </row>
     <row r="41" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="42" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="43" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="44" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="45" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1391,7 +1391,7 @@
     </row>
     <row r="49" spans="1:1" ht="85" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="50" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1401,7 +1401,7 @@
     </row>
     <row r="51" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="52" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1416,7 +1416,7 @@
     </row>
     <row r="54" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="55" spans="1:1" ht="34" x14ac:dyDescent="0.2">
@@ -1426,17 +1426,17 @@
     </row>
     <row r="56" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="57" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="58" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
     </row>
     <row r="59" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1456,7 +1456,7 @@
     </row>
     <row r="62" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
     </row>
     <row r="63" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1476,27 +1476,27 @@
     </row>
     <row r="66" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
     </row>
     <row r="67" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
     </row>
     <row r="68" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
     </row>
     <row r="69" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
     </row>
     <row r="70" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="71" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1511,17 +1511,17 @@
     </row>
     <row r="73" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="74" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="75" spans="1:1" ht="153" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="76" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1531,42 +1531,42 @@
     </row>
     <row r="77" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="78" spans="1:1" ht="119" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="79" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A79" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="80" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="81" spans="1:1" ht="119" x14ac:dyDescent="0.2">
       <c r="A81" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="82" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="83" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A83" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="84" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A84" s="2" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="85" spans="1:1" ht="34" x14ac:dyDescent="0.2">
@@ -1581,17 +1581,17 @@
     </row>
     <row r="87" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="88" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="89" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="90" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1601,12 +1601,12 @@
     </row>
     <row r="91" spans="1:1" ht="136" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="92" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="93" spans="1:1" ht="17" x14ac:dyDescent="0.2">
@@ -1624,7 +1624,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="96" spans="1:1" ht="34" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:1" ht="51" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
         <v>7</v>
       </c>
@@ -1636,12 +1636,12 @@
     </row>
     <row r="98" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="99" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="100" spans="1:1" ht="68" x14ac:dyDescent="0.2">
@@ -1656,22 +1656,22 @@
     </row>
     <row r="102" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A102" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="103" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A103" s="2" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
     </row>
     <row r="104" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A104" s="2" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.2">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A105" s="2" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -1690,1784 +1690,1784 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:3" s="1" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>71</v>
-      </c>
       <c r="C2" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="18" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="19" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="20" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="21" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="22" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" spans="1:3" s="1" customFormat="1" ht="409" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="24" spans="1:3" s="1" customFormat="1" ht="238" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="26" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="27" spans="1:3" s="1" customFormat="1" ht="68" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="29" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="30" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="31" spans="1:3" s="1" customFormat="1" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="32" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="33" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="34" spans="1:3" s="1" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="35" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="36" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="37" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="38" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="39" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="40" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="41" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="42" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="43" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="44" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="45" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="46" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="47" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="48" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="49" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="50" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="51" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="52" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="53" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="54" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="55" spans="1:3" s="1" customFormat="1" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B55" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B55" s="2" t="s">
-        <v>118</v>
-      </c>
       <c r="C55" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="56" spans="1:3" s="1" customFormat="1" ht="238" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="57" spans="1:3" s="1" customFormat="1" ht="221" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="58" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="59" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="60" spans="1:3" s="1" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="61" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="62" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="63" spans="1:3" s="1" customFormat="1" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="64" spans="1:3" s="1" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="65" spans="1:3" s="1" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="66" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="67" spans="1:3" s="1" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="68" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="69" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="70" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="71" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="72" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="73" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="74" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="75" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="76" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="77" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="78" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="79" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="80" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="81" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="82" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="83" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="84" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="85" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="86" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="87" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="88" spans="1:3" s="1" customFormat="1" ht="170" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B88" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="B88" s="2" t="s">
-        <v>132</v>
-      </c>
       <c r="C88" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="89" spans="1:3" s="1" customFormat="1" ht="238" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="90" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="91" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="92" spans="1:3" s="1" customFormat="1" ht="68" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="93" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="94" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="95" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="96" spans="1:3" s="1" customFormat="1" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="97" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="98" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="99" spans="1:3" s="1" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="100" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="101" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="102" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="103" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="104" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="105" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="106" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="107" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="108" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="109" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="110" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="111" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="112" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="113" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="114" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="115" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="116" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="117" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="118" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="119" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="120" spans="1:3" s="1" customFormat="1" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B120" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="B120" s="2" t="s">
-        <v>138</v>
-      </c>
       <c r="C120" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="121" spans="1:3" s="1" customFormat="1" ht="238" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="122" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="123" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="124" spans="1:3" s="1" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="125" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="126" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="127" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="128" spans="1:3" s="1" customFormat="1" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="129" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="130" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="131" spans="1:3" s="1" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="132" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B132" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="133" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B133" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="134" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B134" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="135" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B135" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="136" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="137" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="138" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B138" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="139" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="140" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B140" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="141" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="142" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B142" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="143" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="144" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="145" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B145" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="146" spans="1:3" s="1" customFormat="1" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="147" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B147" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="148" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B148" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="149" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="150" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B150" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="151" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="152" spans="1:3" s="1" customFormat="1" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B152" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B152" s="2" t="s">
-        <v>144</v>
-      </c>
       <c r="C152" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="153" spans="1:3" s="1" customFormat="1" ht="238" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="154" spans="1:3" s="1" customFormat="1" ht="221" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="155" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B155" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="156" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="157" spans="1:3" s="1" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="158" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="159" spans="1:3" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="160" spans="1:3" s="1" customFormat="1" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="161" spans="1:3" s="1" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="162" spans="1:3" s="1" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>